<commit_message>
Weather icons and wind direction
</commit_message>
<xml_diff>
--- a/examples/WeatherClient API Field Mapping.xlsx
+++ b/examples/WeatherClient API Field Mapping.xlsx
@@ -1,20 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10302"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10308"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nick/dev/sc_utility/examples/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{499C63BA-DCA8-0A4C-8624-B28EA497AA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD28422E-250C-8443-8433-09A04625E70C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-47960" yWindow="6020" windowWidth="39060" windowHeight="30740" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-30860" yWindow="6020" windowWidth="21960" windowHeight="30740" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Providers" sheetId="1" r:id="rId1"/>
     <sheet name="Field Mapping" sheetId="2" r:id="rId2"/>
+    <sheet name="Icons" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -34,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="311" uniqueCount="233">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="355" uniqueCount="266">
   <si>
     <t>WeatherClient API Field Mapping</t>
   </si>
@@ -733,13 +734,112 @@
   </si>
   <si>
     <t>daily[].rain.all</t>
+  </si>
+  <si>
+    <t>thunderstorm</t>
+  </si>
+  <si>
+    <t>heavy rain</t>
+  </si>
+  <si>
+    <t>shower rain</t>
+  </si>
+  <si>
+    <t>drizzle</t>
+  </si>
+  <si>
+    <t>snow</t>
+  </si>
+  <si>
+    <t>sleet</t>
+  </si>
+  <si>
+    <t>fog</t>
+  </si>
+  <si>
+    <t>mist</t>
+  </si>
+  <si>
+    <t>haze</t>
+  </si>
+  <si>
+    <t>smoke</t>
+  </si>
+  <si>
+    <t>sand</t>
+  </si>
+  <si>
+    <t>dust</t>
+  </si>
+  <si>
+    <t>overcast</t>
+  </si>
+  <si>
+    <t>broken clouds</t>
+  </si>
+  <si>
+    <t>scattered clouds</t>
+  </si>
+  <si>
+    <t>partly cloudy</t>
+  </si>
+  <si>
+    <t>few clouds</t>
+  </si>
+  <si>
+    <t>mainly clear</t>
+  </si>
+  <si>
+    <t>clear</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> ⛈️</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 🌧️</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 🌦️</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> ❄️</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 🌨️</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 🌫️</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> ☁️</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> ⛅</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 🌤️</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> ☀️</t>
+  </si>
+  <si>
+    <t>Condition</t>
+  </si>
+  <si>
+    <t>Icon</t>
+  </si>
+  <si>
+    <t>💧</t>
+  </si>
+  <si>
+    <t>raindrop</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -792,8 +892,22 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="36"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="0"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -812,6 +926,18 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="1" tint="0.34998626667073579"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.14999847407452621"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -827,7 +953,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="2"/>
@@ -872,6 +998,22 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hyperlink" xfId="2" builtinId="8"/>
@@ -879,6 +1021,12 @@
     <cellStyle name="Title" xfId="1" builtinId="15"/>
   </cellStyles>
   <dxfs count="17">
+    <dxf>
+      <alignment horizontal="general" vertical="center" wrapText="1"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" wrapText="1"/>
+    </dxf>
     <dxf>
       <alignment horizontal="general" vertical="center"/>
     </dxf>
@@ -910,12 +1058,6 @@
       <alignment horizontal="general" vertical="center"/>
     </dxf>
     <dxf>
-      <alignment horizontal="general" vertical="center" wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" wrapText="1"/>
-    </dxf>
-    <dxf>
       <alignment horizontal="general" vertical="center"/>
     </dxf>
     <dxf>
@@ -944,33 +1086,33 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="Table2" displayName="Table2" ref="A5:F13" totalsRowShown="0" dataDxfId="16">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="Table2" displayName="Table2" ref="A5:F13" totalsRowShown="0" dataDxfId="6">
   <autoFilter ref="A5:F13" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="Provider" dataDxfId="15"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0100-000005000000}" name="Service" dataDxfId="14"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="Type" dataDxfId="13"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0100-000003000000}" name="Intervals" dataDxfId="12"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0100-000004000000}" name="API Documentation" dataDxfId="11"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0100-000006000000}" name="Sample API Call" dataDxfId="10"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="Provider" dataDxfId="5"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0100-000005000000}" name="Service" dataDxfId="4"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="Type" dataDxfId="3"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0100-000003000000}" name="Intervals" dataDxfId="2"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0100-000004000000}" name="API Documentation" dataDxfId="1"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0100-000006000000}" name="Sample API Call" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A4:I39" totalsRowShown="0" dataDxfId="9">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A4:I39" totalsRowShown="0" dataDxfId="16">
   <autoFilter ref="A4:I39" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="WeatherClient Field" dataDxfId="8"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="OWM v3: Current" dataDxfId="7"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="OWM v3: Hourly" dataDxfId="6"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="OWM v3: Daily" dataDxfId="5"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="OWM v2.5: Current" dataDxfId="4"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="OWM v2.5: Hourly" dataDxfId="3"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="OpenMeteo Current" dataDxfId="2"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="OpenMeteo Hourly" dataDxfId="1"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="OpenMeteo Daily" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="WeatherClient Field" dataDxfId="15"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="OWM v3: Current" dataDxfId="14"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="OWM v3: Hourly" dataDxfId="13"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="OWM v3: Daily" dataDxfId="12"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="OWM v2.5: Current" dataDxfId="11"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="OWM v2.5: Hourly" dataDxfId="10"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="OpenMeteo Current" dataDxfId="9"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="OpenMeteo Hourly" dataDxfId="8"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="OpenMeteo Daily" dataDxfId="7"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2655,4 +2797,200 @@
     <tablePart r:id="rId3"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F21BF93E-4194-9C48-BB5D-4D748A9DA7B2}">
+  <dimension ref="A1:B24"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="23.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.83203125" style="23"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A1" s="18" t="s">
+        <v>262</v>
+      </c>
+      <c r="B1" s="22" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" s="4" customFormat="1" ht="47" x14ac:dyDescent="0.2">
+      <c r="A2" s="19" t="s">
+        <v>233</v>
+      </c>
+      <c r="B2" s="20" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" s="4" customFormat="1" ht="47" x14ac:dyDescent="0.2">
+      <c r="A3" s="19" t="s">
+        <v>234</v>
+      </c>
+      <c r="B3" s="20" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" s="4" customFormat="1" ht="47" x14ac:dyDescent="0.2">
+      <c r="A4" s="19" t="s">
+        <v>235</v>
+      </c>
+      <c r="B4" s="20" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" s="4" customFormat="1" ht="47" x14ac:dyDescent="0.2">
+      <c r="A5" s="19" t="s">
+        <v>162</v>
+      </c>
+      <c r="B5" s="20" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" s="4" customFormat="1" ht="47" x14ac:dyDescent="0.2">
+      <c r="A6" s="19" t="s">
+        <v>236</v>
+      </c>
+      <c r="B6" s="20" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" s="4" customFormat="1" ht="47" x14ac:dyDescent="0.2">
+      <c r="A7" s="19" t="s">
+        <v>237</v>
+      </c>
+      <c r="B7" s="20" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" s="4" customFormat="1" ht="47" x14ac:dyDescent="0.2">
+      <c r="A8" s="19" t="s">
+        <v>238</v>
+      </c>
+      <c r="B8" s="20" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" s="4" customFormat="1" ht="47" x14ac:dyDescent="0.2">
+      <c r="A9" s="19" t="s">
+        <v>239</v>
+      </c>
+      <c r="B9" s="20" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" s="4" customFormat="1" ht="47" x14ac:dyDescent="0.2">
+      <c r="A10" s="19" t="s">
+        <v>240</v>
+      </c>
+      <c r="B10" s="20" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" s="4" customFormat="1" ht="47" x14ac:dyDescent="0.2">
+      <c r="A11" s="19" t="s">
+        <v>241</v>
+      </c>
+      <c r="B11" s="20" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" s="4" customFormat="1" ht="47" x14ac:dyDescent="0.2">
+      <c r="A12" s="19" t="s">
+        <v>242</v>
+      </c>
+      <c r="B12" s="20" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" s="4" customFormat="1" ht="47" x14ac:dyDescent="0.2">
+      <c r="A13" s="19" t="s">
+        <v>243</v>
+      </c>
+      <c r="B13" s="20" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" s="4" customFormat="1" ht="47" x14ac:dyDescent="0.2">
+      <c r="A14" s="19" t="s">
+        <v>244</v>
+      </c>
+      <c r="B14" s="20" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" s="4" customFormat="1" ht="47" x14ac:dyDescent="0.2">
+      <c r="A15" s="19" t="s">
+        <v>245</v>
+      </c>
+      <c r="B15" s="20" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" s="4" customFormat="1" ht="47" x14ac:dyDescent="0.2">
+      <c r="A16" s="19" t="s">
+        <v>246</v>
+      </c>
+      <c r="B16" s="20" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" s="4" customFormat="1" ht="47" x14ac:dyDescent="0.2">
+      <c r="A17" s="19" t="s">
+        <v>247</v>
+      </c>
+      <c r="B17" s="20" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" s="4" customFormat="1" ht="47" x14ac:dyDescent="0.2">
+      <c r="A18" s="19" t="s">
+        <v>248</v>
+      </c>
+      <c r="B18" s="20" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" s="4" customFormat="1" ht="47" x14ac:dyDescent="0.2">
+      <c r="A19" s="19" t="s">
+        <v>249</v>
+      </c>
+      <c r="B19" s="20" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" s="4" customFormat="1" ht="47" x14ac:dyDescent="0.2">
+      <c r="A20" s="19" t="s">
+        <v>250</v>
+      </c>
+      <c r="B20" s="20" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" s="4" customFormat="1" ht="47" x14ac:dyDescent="0.2">
+      <c r="A21" s="19" t="s">
+        <v>251</v>
+      </c>
+      <c r="B21" s="20" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" s="4" customFormat="1" ht="47" x14ac:dyDescent="0.2">
+      <c r="A22" s="19" t="s">
+        <v>265</v>
+      </c>
+      <c r="B22" s="20" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="47" x14ac:dyDescent="0.2">
+      <c r="B23" s="21"/>
+    </row>
+    <row r="24" spans="1:2" ht="47" x14ac:dyDescent="0.2">
+      <c r="B24" s="21"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>